<commit_message>
chore(data): add new event types to the operations sheet
Merge three event types from a working copy of the sheet:
MicrosoftTodo TaskRead, SharePoint SiteCollectionAdminRemoved, and
OneDrive TeamsMeetingRecordingUploaded.

Also keep the 14 event types playbook runs appended since the last
commit, including the DLP rule matches, PlanListRead, and the
SharePoint and OneDrive file and sharing-link operations.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/UALAllOperations.xlsx
+++ b/Data/UALAllOperations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2434" uniqueCount="2434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2442" uniqueCount="2442">
   <si>
     <t>Risk</t>
   </si>
@@ -7322,6 +7322,30 @@
   </si>
   <si>
     <t>Set-MailboxJunkEmailConfiguration</t>
+  </si>
+  <si>
+    <t>ComplianceDLPSharePoint</t>
+  </si>
+  <si>
+    <t>DLPRuleMatch</t>
+  </si>
+  <si>
+    <t>ComplianceDLPExchange</t>
+  </si>
+  <si>
+    <t>DlpRuleMatch</t>
+  </si>
+  <si>
+    <t>Planner</t>
+  </si>
+  <si>
+    <t>PlannerPlanList</t>
+  </si>
+  <si>
+    <t>FileUploadedPartial</t>
+  </si>
+  <si>
+    <t>TeamsMeetingRecordingUploaded</t>
   </si>
 </sst>
 </file>
@@ -7908,8 +7932,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G962" totalsRowShown="0">
-  <autoFilter ref="A1:G961" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G979" totalsRowShown="0">
+  <autoFilter ref="A1:G976" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G835">
     <sortCondition ref="D2:D835"/>
   </sortState>
@@ -8243,7 +8267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207B3246-3E1F-4883-B5B7-F0312ED8EA41}">
-  <dimension ref="A1:G962"/>
+  <dimension ref="A1:G979"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8.140625" customWidth="1"/>
@@ -19324,6 +19348,193 @@
       </c>
       <c r="D962" s="0" t="s">
         <v>2433</v>
+      </c>
+    </row>
+    <row r="963">
+      <c r="B963" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C963" s="0" t="s">
+        <v>2434</v>
+      </c>
+      <c r="D963" s="0" t="s">
+        <v>2435</v>
+      </c>
+    </row>
+    <row r="964">
+      <c r="B964" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="C964" s="0" t="s">
+        <v>2436</v>
+      </c>
+      <c r="D964" s="0" t="s">
+        <v>2437</v>
+      </c>
+    </row>
+    <row r="965">
+      <c r="B965" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C965" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D965" s="0" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="966">
+      <c r="B966" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C966" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D966" s="0" t="s">
+        <v>1732</v>
+      </c>
+    </row>
+    <row r="967">
+      <c r="B967" s="0" t="s">
+        <v>2438</v>
+      </c>
+      <c r="C967" s="0" t="s">
+        <v>2439</v>
+      </c>
+      <c r="D967" s="0" t="s">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="968">
+      <c r="B968" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C968" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D968" s="0" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="B969" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C969" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D969" s="0" t="s">
+        <v>1203</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="B970" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C970" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D970" s="0" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="B971" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C971" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D971" s="0" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="B972" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C972" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D972" s="0" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="973">
+      <c r="B973" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C973" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D973" s="0" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="974">
+      <c r="B974" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C974" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D974" s="0" t="s">
+        <v>2440</v>
+      </c>
+    </row>
+    <row r="975">
+      <c r="B975" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C975" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D975" s="0" t="s">
+        <v>1732</v>
+      </c>
+    </row>
+    <row r="976">
+      <c r="B976" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C976" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D976" s="0" t="s">
+        <v>2402</v>
+      </c>
+    </row>
+    <row r="977">
+      <c r="B977" s="0" t="s">
+        <v>2380</v>
+      </c>
+      <c r="C977" s="0" t="s">
+        <v>2381</v>
+      </c>
+      <c r="D977" s="0" t="s">
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="978">
+      <c r="B978" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C978" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D978" s="0" t="s">
+        <v>1898</v>
+      </c>
+    </row>
+    <row r="979">
+      <c r="B979" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C979" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D979" s="0" t="s">
+        <v>2441</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
build: prepare release 2.12.2
Rebuild the module and regenerate the command help. Add automatic
replies to the Show-IRTMailbox entry in the user investigation guide,
and add the 2.12.2 changelog section.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/UALAllOperations.xlsx
+++ b/Data/UALAllOperations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2442" uniqueCount="2442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2447" uniqueCount="2447">
   <si>
     <t>Risk</t>
   </si>
@@ -7346,6 +7346,21 @@
   </si>
   <si>
     <t>TeamsMeetingRecordingUploaded</t>
+  </si>
+  <si>
+    <t>Remove-MailContact</t>
+  </si>
+  <si>
+    <t>Set-MailContact</t>
+  </si>
+  <si>
+    <t>New-MailContact</t>
+  </si>
+  <si>
+    <t>Hard Delete user.</t>
+  </si>
+  <si>
+    <t>Set user manager.</t>
   </si>
 </sst>
 </file>
@@ -7932,8 +7947,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G979" totalsRowShown="0">
-  <autoFilter ref="A1:G976" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G985" totalsRowShown="0">
+  <autoFilter ref="A1:G979" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G835">
     <sortCondition ref="D2:D835"/>
   </sortState>
@@ -8267,7 +8282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207B3246-3E1F-4883-B5B7-F0312ED8EA41}">
-  <dimension ref="A1:G979"/>
+  <dimension ref="A1:G985"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8.140625" customWidth="1"/>
@@ -19535,6 +19550,72 @@
       </c>
       <c r="D979" s="0" t="s">
         <v>2441</v>
+      </c>
+    </row>
+    <row r="980">
+      <c r="B980" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="C980" s="0" t="s">
+        <v>594</v>
+      </c>
+      <c r="D980" s="0" t="s">
+        <v>2442</v>
+      </c>
+    </row>
+    <row r="981">
+      <c r="B981" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="C981" s="0" t="s">
+        <v>594</v>
+      </c>
+      <c r="D981" s="0" t="s">
+        <v>2443</v>
+      </c>
+    </row>
+    <row r="982">
+      <c r="B982" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="C982" s="0" t="s">
+        <v>594</v>
+      </c>
+      <c r="D982" s="0" t="s">
+        <v>2444</v>
+      </c>
+    </row>
+    <row r="983">
+      <c r="B983" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C983" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D983" s="0" t="s">
+        <v>2445</v>
+      </c>
+    </row>
+    <row r="984">
+      <c r="B984" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C984" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D984" s="0" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="985">
+      <c r="B985" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C985" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D985" s="0" t="s">
+        <v>2446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>